<commit_message>
fix(calculators): corrected crop input units, updated equations in 5.1, and amended test sheets
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/5.1-inorganic-fertiliser.xlsx
+++ b/packages/calculators/src/modules/test/5.1-inorganic-fertiliser.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/scope1/5-fertiliser/tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A73A0EAF-30E1-4A46-B269-F630AF86BD48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A67C6A3-978A-2F4C-AF7A-67A4C6C55D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51460" yWindow="25620" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
+    <workbookView xWindow="33600" yWindow="-3000" windowWidth="28800" windowHeight="15940" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="5.1.1.1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="60">
   <si>
     <t>MNjf</t>
   </si>
@@ -310,8 +310,11 @@
     <t>Calcium ammonium nitrate (CAN)</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">𝐸𝐹 </t>
+    <t>Monoammonium Phosphate (MAP)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">𝐸 </t>
     </r>
     <r>
       <rPr>
@@ -320,7 +323,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">𝑓𝑗=𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑚𝑎𝑖𝑧𝑒,𝑁2𝑂 </t>
+      <t xml:space="preserve">𝑗𝑓,𝐶𝑂2 </t>
     </r>
     <r>
       <rPr>
@@ -329,7 +332,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">= −0.1474 + (0.0061 × 𝑁 </t>
+      <t xml:space="preserve">= 𝑀𝑈 </t>
     </r>
     <r>
       <rPr>
@@ -338,7 +341,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">𝑓𝑗=𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑚𝑎𝑖𝑧𝑒 </t>
+      <t xml:space="preserve">𝑗𝑓 </t>
     </r>
     <r>
       <rPr>
@@ -347,12 +350,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">𝐸𝐹 </t>
+      <t xml:space="preserve">× 𝐸𝐹 </t>
     </r>
     <r>
       <rPr>
@@ -361,7 +359,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">𝑓𝑗=𝑛𝑜𝑛𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑔𝑟𝑎𝑖𝑛𝑠,𝑁2𝑂 </t>
+      <t>𝑢𝑟𝑒𝑎,𝐶𝑂2</t>
     </r>
     <r>
       <rPr>
@@ -370,7 +368,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">= −0.0781 + (0.0075 × 𝑁 </t>
+      <t xml:space="preserve"> × 𝐶</t>
     </r>
     <r>
       <rPr>
@@ -379,7 +377,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>𝑓𝑗=𝑛𝑜𝑛𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑔𝑟𝑎𝑖𝑛𝑠</t>
+      <t xml:space="preserve">𝐶𝑂2 </t>
     </r>
     <r>
       <rPr>
@@ -388,15 +386,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <t>Monoammonium Phosphate (MAP)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">𝐸 </t>
+      <t>× 10</t>
     </r>
     <r>
       <rPr>
@@ -405,7 +395,33 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">𝑗𝑓,𝐶𝑂2 </t>
+      <t>−3</t>
+    </r>
+  </si>
+  <si>
+    <t>EjfCO2</t>
+  </si>
+  <si>
+    <t>Cco2</t>
+  </si>
+  <si>
+    <t>EFureaco2</t>
+  </si>
+  <si>
+    <t>Mujf</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">𝑀𝑈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">𝑗𝑓 </t>
     </r>
     <r>
       <rPr>
@@ -414,7 +430,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">= 𝑀𝑈 </t>
+      <t xml:space="preserve">= 𝑇𝑀 </t>
     </r>
     <r>
       <rPr>
@@ -432,7 +448,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">× 𝐸𝐹 </t>
+      <t xml:space="preserve">× 𝐹𝑈 </t>
     </r>
     <r>
       <rPr>
@@ -441,104 +457,6 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>𝑢𝑟𝑒𝑎,𝐶𝑂2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> × 𝐶</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝐶𝑂2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>× 10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>−3</t>
-    </r>
-  </si>
-  <si>
-    <t>EjfCO2</t>
-  </si>
-  <si>
-    <t>Cco2</t>
-  </si>
-  <si>
-    <t>EFureaco2</t>
-  </si>
-  <si>
-    <t>Mujf</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">𝑀𝑈 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑗𝑓 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">= 𝑇𝑀 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑗𝑓 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">× 𝐹𝑈 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
       <t>𝑓</t>
     </r>
   </si>
@@ -553,14 +471,30 @@
   </si>
   <si>
     <t>Constants</t>
+  </si>
+  <si>
+    <t>Total mass applied (kg)</t>
+  </si>
+  <si>
+    <t>𝐸𝐹𝑓𝑗=𝑛𝑜𝑛𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑔𝑟𝑎𝑖𝑛𝑠,𝑁2𝑂 = (0.0781 + (0.0075 × 𝑁𝑓𝑗=𝑛𝑜𝑛𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑔𝑟𝑎𝑖𝑛𝑠)) × 10−2</t>
+  </si>
+  <si>
+    <t>𝐸𝐹𝑓𝑗=𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑚𝑎𝑖𝑧𝑒,𝑁2𝑂 = (−0.1474 + (0.0061 × 𝑁𝑓𝑗=𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑚𝑎𝑖𝑧𝑒 )) × 10−2</t>
+  </si>
+  <si>
+    <t>(0.29 + (0.007(𝑒^0.037×𝑁𝑓𝑗=𝑐𝑜𝑡𝑡𝑜𝑛 − 1)) / 𝑁𝑓𝑗=𝑐𝑜𝑡𝑡𝑜𝑛) × 10−2 (Capped at 0.0183)</t>
+  </si>
+  <si>
+    <t>NOTE: I've removed the '0.01' term from below because I believe it is a mistake, confirmation of this is still pending.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="0.00000000"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
+    <numFmt numFmtId="165" formatCode="0.0000000"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -643,21 +577,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -995,15 +929,16 @@
   <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" style="3" customWidth="1"/>
     <col min="2" max="3" width="26.6640625" customWidth="1"/>
     <col min="6" max="6" width="16.5" customWidth="1"/>
-    <col min="12" max="12" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -1015,28 +950,28 @@
     </row>
     <row r="2" spans="1:15">
       <c r="D2" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="I2" s="1"/>
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="17">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>5</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G3" t="s">
@@ -1051,15 +986,15 @@
       <c r="K3" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="L3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="N3" s="11" t="s">
-        <v>56</v>
+      <c r="N3" s="9" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="17">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B4" t="s">
@@ -1076,8 +1011,8 @@
         <v>0.46</v>
       </c>
       <c r="G4">
-        <f>D4/C4</f>
-        <v>0.5</v>
+        <f t="shared" ref="G4:G22" si="0">IF(ISBLANK(C4), "", (IF(ISNUMBER(F4), F4, E4)*D4)/C4)</f>
+        <v>0.23</v>
       </c>
       <c r="I4">
         <f>IF(ISBLANK(B4), "", IF(ISNUMBER(F4), F4*D4, E4*D4))</f>
@@ -1091,7 +1026,7 @@
         <f>$O$4</f>
         <v>1.5714285714285714</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="11">
         <f>I4*J4*K4/1000</f>
         <v>2.5300000000000002E-4</v>
       </c>
@@ -1104,7 +1039,7 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="17">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B5" t="s">
@@ -1117,12 +1052,12 @@
         <v>40</v>
       </c>
       <c r="E5">
-        <f t="shared" ref="E5:E20" si="0">IF(ISBLANK(B5), "", VLOOKUP(B5,$N$24:$O$30, 2, FALSE))</f>
+        <f t="shared" ref="E5:E19" si="1">IF(ISBLANK(B5), "", VLOOKUP(B5,$N$24:$O$30, 2, FALSE))</f>
         <v>0.18</v>
       </c>
       <c r="G5">
-        <f t="shared" ref="G5" si="1">D5/C5</f>
-        <v>0.4</v>
+        <f t="shared" si="0"/>
+        <v>7.1999999999999995E-2</v>
       </c>
       <c r="I5">
         <f t="shared" ref="I5:I24" si="2">IF(ISBLANK(B5), "", IF(ISNUMBER(F5), F5*D5, E5*D5))</f>
@@ -1155,15 +1090,15 @@
         <v>30</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.21</v>
       </c>
       <c r="F6">
         <v>0.25</v>
       </c>
       <c r="G6">
-        <f>IF(ISBLANK(C6), "", D6/C6)</f>
-        <v>0.3</v>
+        <f t="shared" si="0"/>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="I6">
         <f t="shared" si="2"/>
@@ -1187,11 +1122,11 @@
     </row>
     <row r="7" spans="1:15">
       <c r="E7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G7" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <f t="shared" ref="G7:G25" si="3">IF(ISBLANK(C7), "", D7/C7)</f>
         <v/>
       </c>
       <c r="I7" t="str">
@@ -1199,11 +1134,11 @@
         <v/>
       </c>
       <c r="K7" t="str">
-        <f t="shared" ref="K6:K20" si="4">IF(ISBLANK(J7), "",$O$4)</f>
+        <f t="shared" ref="K7:K19" si="3">IF(ISBLANK(J7), "",$O$4)</f>
         <v/>
       </c>
       <c r="L7" t="str">
-        <f t="shared" ref="L7:L20" si="5">IF(ISBLANK(A7), "", I7*J7*K7/1000)</f>
+        <f t="shared" ref="L7:L19" si="4">IF(ISBLANK(A7), "", I7*J7*K7/1000)</f>
         <v/>
       </c>
       <c r="N7" s="2" t="s">
@@ -1215,11 +1150,11 @@
     </row>
     <row r="8" spans="1:15">
       <c r="E8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G8" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G8" t="str">
-        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="I8" t="str">
@@ -1227,11 +1162,11 @@
         <v/>
       </c>
       <c r="K8" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L8" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="L8" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="N8" s="2" t="s">
@@ -1242,15 +1177,15 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="17">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G9" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G9" t="str">
-        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="I9" t="str">
@@ -1258,11 +1193,7 @@
         <v/>
       </c>
       <c r="J9" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="L9" t="str">
-        <f>IF(ISBLANK(B9), "", I9*J9*K9/1000)</f>
-        <v/>
+        <v>57</v>
       </c>
       <c r="N9" s="2" t="s">
         <v>23</v>
@@ -1272,7 +1203,7 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="34">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1285,28 +1216,28 @@
         <v>7000</v>
       </c>
       <c r="E10">
+        <f t="shared" si="1"/>
+        <v>0.21</v>
+      </c>
+      <c r="G10">
         <f t="shared" si="0"/>
-        <v>0.21</v>
-      </c>
-      <c r="G10">
-        <f t="shared" si="3"/>
-        <v>35</v>
+        <v>7.35</v>
       </c>
       <c r="I10">
         <f t="shared" si="2"/>
         <v>1470</v>
       </c>
       <c r="J10">
-        <f>-0.1474 + (0.0061 * G10)</f>
-        <v>6.610000000000002E-2</v>
+        <f>(-0.1474 + (0.0061 * G10)) * 10^-2</f>
+        <v>-1.0256500000000001E-3</v>
       </c>
       <c r="K10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.5714285714285714</v>
       </c>
-      <c r="L10" s="6">
-        <f t="shared" si="5"/>
-        <v>0.15269100000000002</v>
+      <c r="L10" s="5">
+        <f>IF(ISBLANK(A10), "", I10*J10*K10/1000)</f>
+        <v>-2.3692515000000003E-3</v>
       </c>
       <c r="N10" s="2" t="s">
         <v>20</v>
@@ -1316,7 +1247,7 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="34">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B11" t="s">
@@ -1329,31 +1260,31 @@
         <v>3000</v>
       </c>
       <c r="E11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.46</v>
       </c>
       <c r="F11">
         <v>0.4</v>
       </c>
       <c r="G11">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>12</v>
       </c>
       <c r="I11">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
       <c r="J11">
-        <f>-0.1474 + (0.0061 * G11)</f>
-        <v>3.5600000000000021E-2</v>
+        <f>(-0.1474 + (0.0061 * G11)) * 10^-2</f>
+        <v>-7.4200000000000004E-4</v>
       </c>
       <c r="K11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.5714285714285714</v>
       </c>
-      <c r="L11" s="6">
-        <f t="shared" ref="L11" si="6">IF(ISBLANK(A11), "", I11*J11*K11/1000)</f>
-        <v>6.713142857142862E-2</v>
+      <c r="L11" s="5">
+        <f t="shared" ref="L11" si="5">IF(ISBLANK(A11), "", I11*J11*K11/1000)</f>
+        <v>-1.3992E-3</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>24</v>
@@ -1364,7 +1295,7 @@
     </row>
     <row r="12" spans="1:15">
       <c r="G12" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="I12" t="str">
@@ -1380,11 +1311,11 @@
     </row>
     <row r="13" spans="1:15">
       <c r="E13" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G13" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="I13" t="str">
@@ -1392,11 +1323,7 @@
         <v/>
       </c>
       <c r="J13" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L13" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+        <v>56</v>
       </c>
       <c r="N13" s="2" t="s">
         <v>26</v>
@@ -1406,7 +1333,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="34">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -1423,16 +1350,16 @@
         <v>0.33700000000000002</v>
       </c>
       <c r="G14">
-        <f t="shared" si="3"/>
-        <v>100</v>
+        <f t="shared" si="0"/>
+        <v>33.700000000000003</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
         <v>1685</v>
       </c>
       <c r="J14">
-        <f>-0.0781 + (0.0075*G14)</f>
-        <v>0.67189999999999994</v>
+        <f>(0.0781 + (0.0075*G14)) * 10^-2</f>
+        <v>3.3085000000000002E-3</v>
       </c>
       <c r="K14">
         <f>IF(ISBLANK(J14), "",$O$4)</f>
@@ -1440,7 +1367,7 @@
       </c>
       <c r="L14">
         <f>IF(ISBLANK(A14), "", I14*J14*K14/1000)</f>
-        <v>1.7790952142857142</v>
+        <v>8.7604353571428591E-3</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>27</v>
@@ -1450,11 +1377,11 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="34">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15">
         <v>20</v>
@@ -1470,16 +1397,16 @@
         <v>0.2</v>
       </c>
       <c r="G15">
-        <f t="shared" si="3"/>
-        <v>150</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="I15">
         <f t="shared" si="2"/>
         <v>600</v>
       </c>
       <c r="J15">
-        <f>-0.0781 + (0.0075*G15)</f>
-        <v>1.0468999999999999</v>
+        <f>(0.0781 + (0.0075*G15)) * 10^-2</f>
+        <v>3.0309999999999998E-3</v>
       </c>
       <c r="K15">
         <f>IF(ISBLANK(J15), "",$O$4)</f>
@@ -1487,7 +1414,7 @@
       </c>
       <c r="L15">
         <f>IF(ISBLANK(A15), "", I15*J15*K15/1000)</f>
-        <v>0.98707714285714276</v>
+        <v>2.8578000000000002E-3</v>
       </c>
       <c r="N15" s="2" t="s">
         <v>28</v>
@@ -1498,7 +1425,7 @@
     </row>
     <row r="16" spans="1:15">
       <c r="G16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="I16" t="str">
@@ -1514,11 +1441,11 @@
     </row>
     <row r="17" spans="1:15">
       <c r="E17" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G17" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G17" t="str">
-        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="I17" t="str">
@@ -1526,11 +1453,11 @@
         <v/>
       </c>
       <c r="K17" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L17" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="L17" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="N17" s="2" t="s">
@@ -1542,58 +1469,56 @@
     </row>
     <row r="18" spans="1:15">
       <c r="E18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G18" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G18" t="str">
-        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="I18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K18" t="str">
+      <c r="J18" t="s">
+        <v>59</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="3"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="L18" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="L18" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="N18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="O18" s="3">
+      <c r="O18" s="10">
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="E19" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G19" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G19" t="str">
-        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="I19" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K19" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="L19" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="J19" t="s">
+        <v>58</v>
       </c>
       <c r="N19" s="2"/>
-      <c r="O19" s="3"/>
+      <c r="O19" s="10"/>
     </row>
     <row r="20" spans="1:15" ht="17">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B20" s="2" t="s">
@@ -1610,16 +1535,16 @@
         <v>0.27</v>
       </c>
       <c r="G20">
-        <f t="shared" si="3"/>
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>4.05</v>
       </c>
       <c r="I20">
         <f t="shared" si="2"/>
         <v>81</v>
       </c>
       <c r="J20">
-        <f>0.01*(0.29 + (0.007*(EXP(0.037*G20) - 1)/G20))</f>
-        <v>2.9034623912622785E-3</v>
+        <f>MIN(((0.29 + (0.007*(EXP(0.037*G20) - 1)/G20)) * 10^-2), 0.0183)</f>
+        <v>2.9027941231225501E-3</v>
       </c>
       <c r="K20">
         <f>IF(ISBLANK(J20), "",$O$4)</f>
@@ -1627,7 +1552,7 @@
       </c>
       <c r="L20">
         <f>IF(ISBLANK(A20), "", I20*J20*K20/1000)</f>
-        <v>3.6956928437352715E-4</v>
+        <v>3.6948422338602751E-4</v>
       </c>
       <c r="N20" s="2" t="s">
         <v>29</v>
@@ -1637,7 +1562,7 @@
       </c>
     </row>
     <row r="21" spans="1:15" ht="17">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -1657,16 +1582,16 @@
         <v>0.5</v>
       </c>
       <c r="G21">
-        <f t="shared" si="3"/>
-        <v>14</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="I21">
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
       <c r="J21">
-        <f>0.01*(0.29 + (0.007*(EXP(0.037*G21) - 1)/G21))</f>
-        <v>2.9033933347810659E-3</v>
+        <f t="shared" ref="J21:J22" si="6">MIN(((0.29 + (0.007*(EXP(0.037*G21) - 1)/G21)) * 10^-2), 0.0183)</f>
+        <v>2.9029563380482803E-3</v>
       </c>
       <c r="K21">
         <f>IF(ISBLANK(J21), "",$O$4)</f>
@@ -1674,7 +1599,7 @@
       </c>
       <c r="L21">
         <f>IF(ISBLANK(A21), "", I21*J21*K21/1000)</f>
-        <v>7.9843316706479318E-4</v>
+        <v>7.9831299296327706E-4</v>
       </c>
       <c r="N21" s="2" t="s">
         <v>32</v>
@@ -1683,24 +1608,80 @@
         <v>1.8E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
-      <c r="G22" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I22" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:15">
-      <c r="G23" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I23" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+    <row r="22" spans="1:15" ht="17">
+      <c r="A22" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22">
+        <v>25</v>
+      </c>
+      <c r="D22">
+        <v>22200</v>
+      </c>
+      <c r="E22">
+        <f>IF(ISBLANK(B22), "", VLOOKUP(B22,$N$24:$O$30, 2, FALSE))</f>
+        <v>0.33700000000000002</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>299.25600000000003</v>
+      </c>
+      <c r="I22">
+        <f t="shared" ref="I22" si="7">IF(ISBLANK(B22), "", IF(ISNUMBER(F22), F22*D22, E22*D22))</f>
+        <v>7481.4000000000005</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="6"/>
+        <v>1.7957813628911919E-2</v>
+      </c>
+      <c r="K22">
+        <f>IF(ISBLANK(J22), "",$O$4)</f>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="L22">
+        <f>IF(ISBLANK(A22), "", I22*J22*K22/1000)</f>
+        <v>0.21112077938810828</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="17">
+      <c r="A23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23">
+        <v>25</v>
+      </c>
+      <c r="D23">
+        <v>22300</v>
+      </c>
+      <c r="E23">
+        <f>IF(ISBLANK(B23), "", VLOOKUP(B23,$N$24:$O$30, 2, FALSE))</f>
+        <v>0.33700000000000002</v>
+      </c>
+      <c r="G23">
+        <f>IF(ISBLANK(C23), "", (IF(ISNUMBER(F23), F23, E23)*D23)/C23)</f>
+        <v>300.60400000000004</v>
+      </c>
+      <c r="I23">
+        <f t="shared" ref="I23" si="8">IF(ISBLANK(B23), "", IF(ISNUMBER(F23), F23*D23, E23*D23))</f>
+        <v>7515.1</v>
+      </c>
+      <c r="J23">
+        <f t="shared" ref="J23" si="9">MIN(((0.29 + (0.007*(EXP(0.037*G23) - 1)/G23)) * 10^-2), 0.0183)</f>
+        <v>1.83E-2</v>
+      </c>
+      <c r="K23">
+        <f>IF(ISBLANK(J23), "",$O$4)</f>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="L23">
+        <f>IF(ISBLANK(A23), "", I23*J23*K23/1000)</f>
+        <v>0.21611280428571428</v>
       </c>
       <c r="N23" s="2" t="s">
         <v>11</v>
@@ -1708,7 +1689,7 @@
     </row>
     <row r="24" spans="1:15">
       <c r="G24" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="G7:G25" si="10">IF(ISBLANK(C24), "", D24/C24)</f>
         <v/>
       </c>
       <c r="I24" t="str">
@@ -1724,7 +1705,7 @@
     </row>
     <row r="25" spans="1:15">
       <c r="G25" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="N25" s="2" t="s">
@@ -1787,7 +1768,7 @@
   <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" style="3" customWidth="1"/>
     <col min="2" max="3" width="26.6640625" customWidth="1"/>
     <col min="6" max="6" width="16.5" customWidth="1"/>
     <col min="12" max="12" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -1795,14 +1776,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -1816,8 +1797,8 @@
     <row r="4" spans="1:15">
       <c r="I4" s="1"/>
       <c r="L4" s="1"/>
-      <c r="N4" s="11" t="s">
-        <v>56</v>
+      <c r="N4" s="9" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -1828,38 +1809,36 @@
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="17">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="K6" t="s">
-        <v>49</v>
-      </c>
-      <c r="L6" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="17">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B7" t="s">
@@ -1871,8 +1850,6 @@
       <c r="D7">
         <v>50</v>
       </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
       <c r="H7">
         <f>IF(ISBLANK(B7), "", VLOOKUP(B7,$N$27:$O$33, 2, FALSE))</f>
         <v>1</v>
@@ -1894,7 +1871,7 @@
         <v>3.6666666666666667E-2</v>
       </c>
       <c r="N7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="O7">
         <f>44/12</f>
@@ -1902,11 +1879,11 @@
       </c>
     </row>
     <row r="8" spans="1:15" ht="17">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -1914,8 +1891,6 @@
       <c r="D8">
         <v>40</v>
       </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
       <c r="H8">
         <f>IF(ISBLANK(B8), "", VLOOKUP(B8,$N$27:$O$33, 2, FALSE))</f>
         <v>0.35</v>
@@ -1925,15 +1900,15 @@
         <v>14</v>
       </c>
       <c r="J8">
-        <f t="shared" ref="J8:J24" si="0">IF(ISBLANK(A8), "", $O$9)</f>
+        <f t="shared" ref="J8:J11" si="0">IF(ISBLANK(A8), "", $O$9)</f>
         <v>0.2</v>
       </c>
       <c r="K8">
-        <f t="shared" ref="K8:K24" si="1">IF(ISBLANK(A8), "", $O$7)</f>
+        <f t="shared" ref="K8:K11" si="1">IF(ISBLANK(A8), "", $O$7)</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="L8">
-        <f t="shared" ref="L8:L24" si="2">IF(ISBLANK(A8), "", I8*J8*K8/1000)</f>
+        <f t="shared" ref="L8:L11" si="2">IF(ISBLANK(A8), "", I8*J8*K8/1000)</f>
         <v>1.0266666666666667E-2</v>
       </c>
     </row>
@@ -1950,8 +1925,6 @@
       <c r="D9">
         <v>30</v>
       </c>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
       <c r="H9">
         <f>IF(ISBLANK(B9), "", VLOOKUP(B9,$N$27:$O$33, 2, FALSE))</f>
         <v>0</v>
@@ -1973,7 +1946,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O9">
         <v>0.2</v>
@@ -1981,13 +1954,11 @@
     </row>
     <row r="10" spans="1:15">
       <c r="E10" t="str">
-        <f t="shared" ref="E8:E24" si="3">IF(ISBLANK(B10), "", VLOOKUP(B10,$N$27:$O$33, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
+        <f t="shared" ref="E10:E11" si="3">IF(ISBLANK(B10), "", VLOOKUP(B10,$N$27:$O$33, 2, FALSE))</f>
+        <v/>
+      </c>
       <c r="I10" t="str">
-        <f t="shared" ref="I8:I24" si="4">IF(ISBLANK(B10), "", D10*E10)</f>
+        <f t="shared" ref="I10:I11" si="4">IF(ISBLANK(B10), "", D10*E10)</f>
         <v/>
       </c>
       <c r="J10" t="str">
@@ -2010,8 +1981,6 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
       <c r="I11" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2032,96 +2001,70 @@
       <c r="O11" s="2"/>
     </row>
     <row r="12" spans="1:15">
-      <c r="A12" s="5"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
+      <c r="A12" s="4"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
     <row r="13" spans="1:15">
       <c r="B13" s="2"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
     </row>
     <row r="14" spans="1:15">
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>
     <row r="15" spans="1:15">
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
     </row>
     <row r="16" spans="1:15">
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="2"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="2"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
       <c r="N21" s="2"/>
-      <c r="O21" s="3"/>
+      <c r="O21" s="10"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
       <c r="N22" s="2"/>
-      <c r="O22" s="3"/>
+      <c r="O22" s="10"/>
     </row>
     <row r="23" spans="2:15">
       <c r="B23" s="2"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
     </row>
     <row r="24" spans="2:15">
       <c r="B24" s="2"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
     </row>
     <row r="25" spans="2:15">
       <c r="G25" t="str">
-        <f t="shared" ref="G10:G28" si="5">IF(ISBLANK(C25), "", D25/C25)</f>
+        <f t="shared" ref="G25:G28" si="5">IF(ISBLANK(C25), "", D25/C25)</f>
         <v/>
       </c>
       <c r="I25" t="str">
-        <f t="shared" ref="I8:I27" si="6">IF(ISBLANK(B25), "", IF(ISNUMBER(F25), F25*D25, E25*D25))</f>
+        <f t="shared" ref="I25:I27" si="6">IF(ISBLANK(B25), "", IF(ISNUMBER(F25), F25*D25, E25*D25))</f>
         <v/>
       </c>
     </row>
@@ -2135,7 +2078,7 @@
         <v/>
       </c>
       <c r="N26" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="2:15">

</xml_diff>